<commit_message>
fix(neuroforge): update team members for NeuroForge and re-export certificates
</commit_message>
<xml_diff>
--- a/hackathon_participants_certificate_ids.xlsx
+++ b/hackathon_participants_certificate_ids.xlsx
@@ -3707,34 +3707,34 @@
         <v>94</v>
       </c>
       <c r="B95" t="str">
-        <v>CERT-9124B923</v>
+        <v>CERT-4EDFADE5</v>
       </c>
       <c r="C95" t="str">
-        <v>Adyasha Samantray</v>
+        <v>Navam Avaanv</v>
       </c>
       <c r="D95" t="str">
-        <v>NeuroForge</v>
+        <v>logic coders</v>
       </c>
       <c r="E95" t="str">
-        <v>TEAM-2026-0037</v>
+        <v>TEAM-2026-0034</v>
       </c>
       <c r="F95" t="str">
-        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
+        <v>Rishihood University</v>
       </c>
       <c r="G95" t="str">
-        <v>teamnexisedge@gmail.com</v>
+        <v>devsoni3436@gmail.com</v>
       </c>
       <c r="H95" t="str">
-        <v>+91 7875443935</v>
+        <v>+91 9648884888</v>
       </c>
       <c r="I95" t="str">
-        <v>Pending</v>
+        <v>Verified</v>
       </c>
       <c r="J95" t="str">
         <v>2026-09-12</v>
       </c>
       <c r="K95" t="str">
-        <v>9124b923-bf0f-4f34-90d2-bdd228b3c802</v>
+        <v>4edfade5-67df-4f29-9bc8-35071ba6fae2</v>
       </c>
     </row>
     <row r="96">
@@ -3742,34 +3742,34 @@
         <v>95</v>
       </c>
       <c r="B96" t="str">
-        <v>CERT-0921DD78</v>
+        <v>CERT-78B9668B</v>
       </c>
       <c r="C96" t="str">
-        <v>Suhana Mishra</v>
+        <v>Prajan</v>
       </c>
       <c r="D96" t="str">
-        <v>NeuroForge</v>
+        <v>logic coders</v>
       </c>
       <c r="E96" t="str">
-        <v>TEAM-2026-0037</v>
+        <v>TEAM-2026-0034</v>
       </c>
       <c r="F96" t="str">
-        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
+        <v>Rishihood University</v>
       </c>
       <c r="G96" t="str">
-        <v>teamnexisedge@gmail.com</v>
+        <v>devsoni3436@gmail.com</v>
       </c>
       <c r="H96" t="str">
-        <v>+91 7875443935</v>
+        <v>+91 9648884888</v>
       </c>
       <c r="I96" t="str">
-        <v>Pending</v>
+        <v>Verified</v>
       </c>
       <c r="J96" t="str">
         <v>2026-09-12</v>
       </c>
       <c r="K96" t="str">
-        <v>0921dd78-843b-4863-bfae-cb750327a492</v>
+        <v>78b9668b-e682-4240-9253-c3883f176952</v>
       </c>
     </row>
     <row r="97">
@@ -3777,34 +3777,34 @@
         <v>96</v>
       </c>
       <c r="B97" t="str">
-        <v>CERT-3BA3C386</v>
+        <v>CERT-472D9990</v>
       </c>
       <c r="C97" t="str">
-        <v>Shadab Khan</v>
+        <v>Ankit Pardhi</v>
       </c>
       <c r="D97" t="str">
-        <v>NeuroForge</v>
+        <v>Innovate x</v>
       </c>
       <c r="E97" t="str">
-        <v>TEAM-2026-0037</v>
+        <v>TEAM-2026-0033</v>
       </c>
       <c r="F97" t="str">
-        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
+        <v>Jai Narain College of Technology (JNCT), Bhopal, Madhya Pradesh</v>
       </c>
       <c r="G97" t="str">
-        <v>teamnexisedge@gmail.com</v>
+        <v>premkumarrinhayat@gmail.com</v>
       </c>
       <c r="H97" t="str">
-        <v>+91 7875443935</v>
+        <v>+91 9098077536</v>
       </c>
       <c r="I97" t="str">
-        <v>Pending</v>
+        <v>Verified</v>
       </c>
       <c r="J97" t="str">
         <v>2026-09-12</v>
       </c>
       <c r="K97" t="str">
-        <v>3ba3c386-3ba9-4294-8db8-a9d7cf9d5972</v>
+        <v>472d9990-10fc-49f2-9cc0-3602b1b035b8</v>
       </c>
     </row>
     <row r="98">
@@ -3812,10 +3812,10 @@
         <v>97</v>
       </c>
       <c r="B98" t="str">
-        <v>CERT-4EDFADE5</v>
+        <v>CERT-51B619FB</v>
       </c>
       <c r="C98" t="str">
-        <v>Navam Avaanv</v>
+        <v>Dev Soni</v>
       </c>
       <c r="D98" t="str">
         <v>logic coders</v>
@@ -3839,7 +3839,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K98" t="str">
-        <v>4edfade5-67df-4f29-9bc8-35071ba6fae2</v>
+        <v>51b619fb-9955-48c8-82cb-d0666f676042</v>
       </c>
     </row>
     <row r="99">
@@ -3847,25 +3847,25 @@
         <v>98</v>
       </c>
       <c r="B99" t="str">
-        <v>CERT-78B9668B</v>
+        <v>CERT-FCC5CD49</v>
       </c>
       <c r="C99" t="str">
-        <v>Prajan</v>
+        <v>Rushan Advani</v>
       </c>
       <c r="D99" t="str">
-        <v>logic coders</v>
+        <v>quasar</v>
       </c>
       <c r="E99" t="str">
-        <v>TEAM-2026-0034</v>
+        <v>TEAM-2026-0046</v>
       </c>
       <c r="F99" t="str">
         <v>Rishihood University</v>
       </c>
       <c r="G99" t="str">
-        <v>devsoni3436@gmail.com</v>
+        <v>amritanshu.nirjhar@gmail.com</v>
       </c>
       <c r="H99" t="str">
-        <v>+91 9648884888</v>
+        <v>+91 8448325338</v>
       </c>
       <c r="I99" t="str">
         <v>Verified</v>
@@ -3874,7 +3874,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K99" t="str">
-        <v>78b9668b-e682-4240-9253-c3883f176952</v>
+        <v>fcc5cd49-2f92-4a8f-aebb-d642cd29a4d3</v>
       </c>
     </row>
     <row r="100">
@@ -3882,25 +3882,25 @@
         <v>99</v>
       </c>
       <c r="B100" t="str">
-        <v>CERT-472D9990</v>
+        <v>CERT-05840BE8</v>
       </c>
       <c r="C100" t="str">
-        <v>Ankit Pardhi</v>
+        <v>Sahaj Choukhani</v>
       </c>
       <c r="D100" t="str">
-        <v>Innovate x</v>
+        <v>quasar</v>
       </c>
       <c r="E100" t="str">
-        <v>TEAM-2026-0033</v>
+        <v>TEAM-2026-0046</v>
       </c>
       <c r="F100" t="str">
-        <v>Jai Narain College of Technology (JNCT), Bhopal, Madhya Pradesh</v>
+        <v>Rishihood University</v>
       </c>
       <c r="G100" t="str">
-        <v>premkumarrinhayat@gmail.com</v>
+        <v>amritanshu.nirjhar@gmail.com</v>
       </c>
       <c r="H100" t="str">
-        <v>+91 9098077536</v>
+        <v>+91 8448325338</v>
       </c>
       <c r="I100" t="str">
         <v>Verified</v>
@@ -3909,7 +3909,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K100" t="str">
-        <v>472d9990-10fc-49f2-9cc0-3602b1b035b8</v>
+        <v>05840be8-2628-48b9-b16d-c1249ecb1f44</v>
       </c>
     </row>
     <row r="101">
@@ -3917,25 +3917,25 @@
         <v>100</v>
       </c>
       <c r="B101" t="str">
-        <v>CERT-51B619FB</v>
+        <v>CERT-B5E6F13B</v>
       </c>
       <c r="C101" t="str">
-        <v>Dev Soni</v>
+        <v>Saksham Verma</v>
       </c>
       <c r="D101" t="str">
-        <v>logic coders</v>
+        <v>Sinisters</v>
       </c>
       <c r="E101" t="str">
-        <v>TEAM-2026-0034</v>
+        <v>TEAM-2026-0048</v>
       </c>
       <c r="F101" t="str">
-        <v>Rishihood University</v>
+        <v>Chhatrapati Shahu Ji Maharaj University (CSJMU), Kanpur</v>
       </c>
       <c r="G101" t="str">
-        <v>devsoni3436@gmail.com</v>
+        <v>sadip1921@gmail.com</v>
       </c>
       <c r="H101" t="str">
-        <v>+91 9648884888</v>
+        <v>+91 9528818624</v>
       </c>
       <c r="I101" t="str">
         <v>Verified</v>
@@ -3944,7 +3944,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K101" t="str">
-        <v>51b619fb-9955-48c8-82cb-d0666f676042</v>
+        <v>b5e6f13b-0be1-4612-812d-9692b2e88b32</v>
       </c>
     </row>
     <row r="102">
@@ -3952,25 +3952,25 @@
         <v>101</v>
       </c>
       <c r="B102" t="str">
-        <v>CERT-FCC5CD49</v>
+        <v>CERT-DC67ED0C</v>
       </c>
       <c r="C102" t="str">
-        <v>Rushan Advani</v>
+        <v>Akhil Soigama</v>
       </c>
       <c r="D102" t="str">
-        <v>quasar</v>
+        <v>NovaMinds</v>
       </c>
       <c r="E102" t="str">
-        <v>TEAM-2026-0046</v>
+        <v>TEAM-2026-0040</v>
       </c>
       <c r="F102" t="str">
-        <v>Rishihood University</v>
+        <v>Dr. Subhash University, Junagadh, Gujarat</v>
       </c>
       <c r="G102" t="str">
-        <v>amritanshu.nirjhar@gmail.com</v>
+        <v>akhilsoigama@gmail.com</v>
       </c>
       <c r="H102" t="str">
-        <v>+91 8448325338</v>
+        <v>+91 9510159304</v>
       </c>
       <c r="I102" t="str">
         <v>Verified</v>
@@ -3979,7 +3979,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K102" t="str">
-        <v>fcc5cd49-2f92-4a8f-aebb-d642cd29a4d3</v>
+        <v>dc67ed0c-eb12-4305-83c4-c445a7357ade</v>
       </c>
     </row>
     <row r="103">
@@ -3987,10 +3987,10 @@
         <v>102</v>
       </c>
       <c r="B103" t="str">
-        <v>CERT-05840BE8</v>
+        <v>CERT-E51F3090</v>
       </c>
       <c r="C103" t="str">
-        <v>Sahaj Choukhani</v>
+        <v>Amritanshu Nirjhar</v>
       </c>
       <c r="D103" t="str">
         <v>quasar</v>
@@ -4014,7 +4014,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K103" t="str">
-        <v>05840be8-2628-48b9-b16d-c1249ecb1f44</v>
+        <v>e51f3090-9eef-4b7e-91b2-9e155d0a1ee5</v>
       </c>
     </row>
     <row r="104">
@@ -4022,10 +4022,10 @@
         <v>103</v>
       </c>
       <c r="B104" t="str">
-        <v>CERT-B5E6F13B</v>
+        <v>CERT-9799D586</v>
       </c>
       <c r="C104" t="str">
-        <v>Saksham Verma</v>
+        <v>Ayush Jaiswal</v>
       </c>
       <c r="D104" t="str">
         <v>Sinisters</v>
@@ -4049,7 +4049,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K104" t="str">
-        <v>b5e6f13b-0be1-4612-812d-9692b2e88b32</v>
+        <v>9799d586-b0b2-453b-ad51-4ad26e2aa25e</v>
       </c>
     </row>
     <row r="105">
@@ -4057,25 +4057,25 @@
         <v>104</v>
       </c>
       <c r="B105" t="str">
-        <v>CERT-DC67ED0C</v>
+        <v>CERT-5FD3CF54</v>
       </c>
       <c r="C105" t="str">
-        <v>Akhil Soigama</v>
+        <v>Gautam Patidar</v>
       </c>
       <c r="D105" t="str">
-        <v>NovaMinds</v>
+        <v>Null and Void</v>
       </c>
       <c r="E105" t="str">
-        <v>TEAM-2026-0040</v>
+        <v>TEAM-2026-0041</v>
       </c>
       <c r="F105" t="str">
-        <v>Dr. Subhash University, Junagadh, Gujarat</v>
+        <v>SAGE University (SAGEU), Indore, Madhya Pradesh</v>
       </c>
       <c r="G105" t="str">
-        <v>akhilsoigama@gmail.com</v>
+        <v>aashutoshkumar2252@gmail.com</v>
       </c>
       <c r="H105" t="str">
-        <v>+91 9510159304</v>
+        <v>+91 9982107838</v>
       </c>
       <c r="I105" t="str">
         <v>Verified</v>
@@ -4084,7 +4084,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K105" t="str">
-        <v>dc67ed0c-eb12-4305-83c4-c445a7357ade</v>
+        <v>5fd3cf54-e2cb-4612-84dd-58507707310c</v>
       </c>
     </row>
     <row r="106">
@@ -4092,25 +4092,25 @@
         <v>105</v>
       </c>
       <c r="B106" t="str">
-        <v>CERT-E51F3090</v>
+        <v>CERT-36182ED1</v>
       </c>
       <c r="C106" t="str">
-        <v>Amritanshu Nirjhar</v>
+        <v>Punit Vithlani</v>
       </c>
       <c r="D106" t="str">
-        <v>quasar</v>
+        <v>NovaMinds</v>
       </c>
       <c r="E106" t="str">
-        <v>TEAM-2026-0046</v>
+        <v>TEAM-2026-0040</v>
       </c>
       <c r="F106" t="str">
-        <v>Rishihood University</v>
+        <v>Dr. Subhash University, Junagadh, Gujarat</v>
       </c>
       <c r="G106" t="str">
-        <v>amritanshu.nirjhar@gmail.com</v>
+        <v>akhilsoigama@gmail.com</v>
       </c>
       <c r="H106" t="str">
-        <v>+91 8448325338</v>
+        <v>+91 9510159304</v>
       </c>
       <c r="I106" t="str">
         <v>Verified</v>
@@ -4119,7 +4119,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K106" t="str">
-        <v>e51f3090-9eef-4b7e-91b2-9e155d0a1ee5</v>
+        <v>36182ed1-ad5a-44ac-bc13-966345a64afb</v>
       </c>
     </row>
     <row r="107">
@@ -4127,25 +4127,25 @@
         <v>106</v>
       </c>
       <c r="B107" t="str">
-        <v>CERT-9799D586</v>
+        <v>CERT-7F2DB5AC</v>
       </c>
       <c r="C107" t="str">
-        <v>Ayush Jaiswal</v>
+        <v>Uday Bhimani</v>
       </c>
       <c r="D107" t="str">
-        <v>Sinisters</v>
+        <v>NovaMinds</v>
       </c>
       <c r="E107" t="str">
-        <v>TEAM-2026-0048</v>
+        <v>TEAM-2026-0040</v>
       </c>
       <c r="F107" t="str">
-        <v>Chhatrapati Shahu Ji Maharaj University (CSJMU), Kanpur</v>
+        <v>Dr. Subhash University, Junagadh, Gujarat</v>
       </c>
       <c r="G107" t="str">
-        <v>sadip1921@gmail.com</v>
+        <v>akhilsoigama@gmail.com</v>
       </c>
       <c r="H107" t="str">
-        <v>+91 9528818624</v>
+        <v>+91 9510159304</v>
       </c>
       <c r="I107" t="str">
         <v>Verified</v>
@@ -4154,7 +4154,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K107" t="str">
-        <v>9799d586-b0b2-453b-ad51-4ad26e2aa25e</v>
+        <v>7f2db5ac-f139-4140-9cfd-c5c7a0e54c9b</v>
       </c>
     </row>
     <row r="108">
@@ -4162,25 +4162,25 @@
         <v>107</v>
       </c>
       <c r="B108" t="str">
-        <v>CERT-5FD3CF54</v>
+        <v>CERT-C528A205</v>
       </c>
       <c r="C108" t="str">
-        <v>Gautam Patidar</v>
+        <v>Sakshi Pandit</v>
       </c>
       <c r="D108" t="str">
-        <v>Null and Void</v>
+        <v>OOPS</v>
       </c>
       <c r="E108" t="str">
-        <v>TEAM-2026-0041</v>
+        <v>TEAM-2026-0043</v>
       </c>
       <c r="F108" t="str">
-        <v>SAGE University (SAGEU), Indore, Madhya Pradesh</v>
+        <v>ABES Engineering College</v>
       </c>
       <c r="G108" t="str">
-        <v>aashutoshkumar2252@gmail.com</v>
+        <v>sakshipandit8742@gmail.com</v>
       </c>
       <c r="H108" t="str">
-        <v>+91 9982107838</v>
+        <v>+91 9927908848</v>
       </c>
       <c r="I108" t="str">
         <v>Verified</v>
@@ -4189,7 +4189,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K108" t="str">
-        <v>5fd3cf54-e2cb-4612-84dd-58507707310c</v>
+        <v>c528a205-6645-40c5-9360-854c46300605</v>
       </c>
     </row>
     <row r="109">
@@ -4197,25 +4197,25 @@
         <v>108</v>
       </c>
       <c r="B109" t="str">
-        <v>CERT-36182ED1</v>
+        <v>CERT-41010441</v>
       </c>
       <c r="C109" t="str">
-        <v>Punit Vithlani</v>
+        <v>Riya</v>
       </c>
       <c r="D109" t="str">
-        <v>NovaMinds</v>
+        <v>OOPS</v>
       </c>
       <c r="E109" t="str">
-        <v>TEAM-2026-0040</v>
+        <v>TEAM-2026-0043</v>
       </c>
       <c r="F109" t="str">
-        <v>Dr. Subhash University, Junagadh, Gujarat</v>
+        <v>ABES Engineering College</v>
       </c>
       <c r="G109" t="str">
-        <v>akhilsoigama@gmail.com</v>
+        <v>sakshipandit8742@gmail.com</v>
       </c>
       <c r="H109" t="str">
-        <v>+91 9510159304</v>
+        <v>+91 9927908848</v>
       </c>
       <c r="I109" t="str">
         <v>Verified</v>
@@ -4224,7 +4224,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K109" t="str">
-        <v>36182ed1-ad5a-44ac-bc13-966345a64afb</v>
+        <v>41010441-9eef-4c14-bfe0-5198f9d9dc2b</v>
       </c>
     </row>
     <row r="110">
@@ -4232,25 +4232,25 @@
         <v>109</v>
       </c>
       <c r="B110" t="str">
-        <v>CERT-7F2DB5AC</v>
+        <v>CERT-D9DA0B3F</v>
       </c>
       <c r="C110" t="str">
-        <v>Uday Bhimani</v>
+        <v>Keerti Sharma</v>
       </c>
       <c r="D110" t="str">
-        <v>NovaMinds</v>
+        <v>PHANTOM BYTE 2.0</v>
       </c>
       <c r="E110" t="str">
-        <v>TEAM-2026-0040</v>
+        <v>TEAM-2026-0044</v>
       </c>
       <c r="F110" t="str">
-        <v>Dr. Subhash University, Junagadh, Gujarat</v>
+        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
       </c>
       <c r="G110" t="str">
-        <v>akhilsoigama@gmail.com</v>
+        <v>keertisharma128@gmail.com</v>
       </c>
       <c r="H110" t="str">
-        <v>+91 9510159304</v>
+        <v>+91 7974120867</v>
       </c>
       <c r="I110" t="str">
         <v>Verified</v>
@@ -4259,7 +4259,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K110" t="str">
-        <v>7f2db5ac-f139-4140-9cfd-c5c7a0e54c9b</v>
+        <v>d9da0b3f-97b5-486e-b627-d05ebf006262</v>
       </c>
     </row>
     <row r="111">
@@ -4267,25 +4267,25 @@
         <v>110</v>
       </c>
       <c r="B111" t="str">
-        <v>CERT-C528A205</v>
+        <v>CERT-F0BB4AE0</v>
       </c>
       <c r="C111" t="str">
-        <v>Sakshi Pandit</v>
+        <v>Astha Goswami</v>
       </c>
       <c r="D111" t="str">
-        <v>OOPS</v>
+        <v>PHANTOM BYTE 2.0</v>
       </c>
       <c r="E111" t="str">
-        <v>TEAM-2026-0043</v>
+        <v>TEAM-2026-0044</v>
       </c>
       <c r="F111" t="str">
-        <v>ABES Engineering College</v>
+        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
       </c>
       <c r="G111" t="str">
-        <v>sakshipandit8742@gmail.com</v>
+        <v>keertisharma128@gmail.com</v>
       </c>
       <c r="H111" t="str">
-        <v>+91 9927908848</v>
+        <v>+91 7974120867</v>
       </c>
       <c r="I111" t="str">
         <v>Verified</v>
@@ -4294,7 +4294,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K111" t="str">
-        <v>c528a205-6645-40c5-9360-854c46300605</v>
+        <v>f0bb4ae0-37a9-4f05-be19-f2d71fe2c7db</v>
       </c>
     </row>
     <row r="112">
@@ -4302,25 +4302,25 @@
         <v>111</v>
       </c>
       <c r="B112" t="str">
-        <v>CERT-41010441</v>
+        <v>CERT-AA22D4B9</v>
       </c>
       <c r="C112" t="str">
-        <v>Riya</v>
+        <v>Samay Sutrakar</v>
       </c>
       <c r="D112" t="str">
-        <v>OOPS</v>
+        <v>PHANTOM BYTE 2.0</v>
       </c>
       <c r="E112" t="str">
-        <v>TEAM-2026-0043</v>
+        <v>TEAM-2026-0044</v>
       </c>
       <c r="F112" t="str">
-        <v>ABES Engineering College</v>
+        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
       </c>
       <c r="G112" t="str">
-        <v>sakshipandit8742@gmail.com</v>
+        <v>keertisharma128@gmail.com</v>
       </c>
       <c r="H112" t="str">
-        <v>+91 9927908848</v>
+        <v>+91 7974120867</v>
       </c>
       <c r="I112" t="str">
         <v>Verified</v>
@@ -4329,7 +4329,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K112" t="str">
-        <v>41010441-9eef-4c14-bfe0-5198f9d9dc2b</v>
+        <v>aa22d4b9-ba27-42d5-8c28-c45e1aa82e04</v>
       </c>
     </row>
     <row r="113">
@@ -4337,25 +4337,25 @@
         <v>112</v>
       </c>
       <c r="B113" t="str">
-        <v>CERT-D9DA0B3F</v>
+        <v>CERT-9D08A880</v>
       </c>
       <c r="C113" t="str">
-        <v>Keerti Sharma</v>
+        <v>Pawan Kushwah</v>
       </c>
       <c r="D113" t="str">
-        <v>PHANTOM BYTE 2.0</v>
+        <v>Null and Void</v>
       </c>
       <c r="E113" t="str">
-        <v>TEAM-2026-0044</v>
+        <v>TEAM-2026-0041</v>
       </c>
       <c r="F113" t="str">
-        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
+        <v>SAGE University (SAGEU), Indore, Madhya Pradesh</v>
       </c>
       <c r="G113" t="str">
-        <v>keertisharma128@gmail.com</v>
+        <v>aashutoshkumar2252@gmail.com</v>
       </c>
       <c r="H113" t="str">
-        <v>+91 7974120867</v>
+        <v>+91 9982107838</v>
       </c>
       <c r="I113" t="str">
         <v>Verified</v>
@@ -4364,7 +4364,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K113" t="str">
-        <v>d9da0b3f-97b5-486e-b627-d05ebf006262</v>
+        <v>9d08a880-681e-479f-9c0b-8ddcae9f4967</v>
       </c>
     </row>
     <row r="114">
@@ -4372,34 +4372,34 @@
         <v>113</v>
       </c>
       <c r="B114" t="str">
-        <v>CERT-F0BB4AE0</v>
+        <v>CERT-9124B923</v>
       </c>
       <c r="C114" t="str">
-        <v>Astha Goswami</v>
+        <v>Samrudhi Chavan</v>
       </c>
       <c r="D114" t="str">
-        <v>PHANTOM BYTE 2.0</v>
+        <v>NeuroForge</v>
       </c>
       <c r="E114" t="str">
-        <v>TEAM-2026-0044</v>
+        <v>TEAM-2026-0037</v>
       </c>
       <c r="F114" t="str">
-        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
+        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
       </c>
       <c r="G114" t="str">
-        <v>keertisharma128@gmail.com</v>
+        <v>teamnexisedge@gmail.com</v>
       </c>
       <c r="H114" t="str">
-        <v>+91 7974120867</v>
+        <v>+91 7875443935</v>
       </c>
       <c r="I114" t="str">
-        <v>Verified</v>
+        <v>Pending</v>
       </c>
       <c r="J114" t="str">
         <v>2026-09-12</v>
       </c>
       <c r="K114" t="str">
-        <v>f0bb4ae0-37a9-4f05-be19-f2d71fe2c7db</v>
+        <v>9124b923-bf0f-4f34-90d2-bdd228b3c802</v>
       </c>
     </row>
     <row r="115">
@@ -4407,25 +4407,25 @@
         <v>114</v>
       </c>
       <c r="B115" t="str">
-        <v>CERT-AA22D4B9</v>
+        <v>CERT-DBB1B88E</v>
       </c>
       <c r="C115" t="str">
-        <v>Samay Sutrakar</v>
+        <v>Deep Jain</v>
       </c>
       <c r="D115" t="str">
-        <v>PHANTOM BYTE 2.0</v>
+        <v>ModelX</v>
       </c>
       <c r="E115" t="str">
-        <v>TEAM-2026-0044</v>
+        <v>TEAM-2026-0035</v>
       </c>
       <c r="F115" t="str">
-        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
+        <v>Institute of Engineering and Science, IPS Academy (IES IPS), Indore</v>
       </c>
       <c r="G115" t="str">
-        <v>keertisharma128@gmail.com</v>
+        <v>deepjain615@gmail.com</v>
       </c>
       <c r="H115" t="str">
-        <v>+91 7974120867</v>
+        <v>+91 9407573955</v>
       </c>
       <c r="I115" t="str">
         <v>Verified</v>
@@ -4434,7 +4434,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K115" t="str">
-        <v>aa22d4b9-ba27-42d5-8c28-c45e1aa82e04</v>
+        <v>dbb1b88e-a042-4d57-8ec9-9819a592f857</v>
       </c>
     </row>
     <row r="116">
@@ -4442,25 +4442,25 @@
         <v>115</v>
       </c>
       <c r="B116" t="str">
-        <v>CERT-9D08A880</v>
+        <v>CERT-F1521375</v>
       </c>
       <c r="C116" t="str">
-        <v>Pawan Kushwah</v>
+        <v>Kartik jaiswal</v>
       </c>
       <c r="D116" t="str">
-        <v>Null and Void</v>
+        <v>Quantum nexus</v>
       </c>
       <c r="E116" t="str">
-        <v>TEAM-2026-0041</v>
+        <v>TEAM-2026-0045</v>
       </c>
       <c r="F116" t="str">
-        <v>SAGE University (SAGEU), Indore, Madhya Pradesh</v>
+        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
       </c>
       <c r="G116" t="str">
-        <v>aashutoshkumar2252@gmail.com</v>
+        <v>kartikjaiswal9565@gmail.com</v>
       </c>
       <c r="H116" t="str">
-        <v>+91 9982107838</v>
+        <v>+91 7828830654</v>
       </c>
       <c r="I116" t="str">
         <v>Verified</v>
@@ -4469,7 +4469,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K116" t="str">
-        <v>9d08a880-681e-479f-9c0b-8ddcae9f4967</v>
+        <v>f1521375-a030-40f5-9c4a-ce9fbb6f6b90</v>
       </c>
     </row>
     <row r="117">
@@ -4477,25 +4477,25 @@
         <v>116</v>
       </c>
       <c r="B117" t="str">
-        <v>CERT-DBB1B88E</v>
+        <v>CERT-4ED0C48E</v>
       </c>
       <c r="C117" t="str">
-        <v>Deep Jain</v>
+        <v>Don Abraham</v>
       </c>
       <c r="D117" t="str">
-        <v>ModelX</v>
+        <v>Quantum nexus</v>
       </c>
       <c r="E117" t="str">
-        <v>TEAM-2026-0035</v>
+        <v>TEAM-2026-0045</v>
       </c>
       <c r="F117" t="str">
-        <v>Institute of Engineering and Science, IPS Academy (IES IPS), Indore</v>
+        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
       </c>
       <c r="G117" t="str">
-        <v>deepjain615@gmail.com</v>
+        <v>kartikjaiswal9565@gmail.com</v>
       </c>
       <c r="H117" t="str">
-        <v>+91 9407573955</v>
+        <v>+91 7828830654</v>
       </c>
       <c r="I117" t="str">
         <v>Verified</v>
@@ -4504,7 +4504,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K117" t="str">
-        <v>dbb1b88e-a042-4d57-8ec9-9819a592f857</v>
+        <v>4ed0c48e-c48e-42de-9bc0-8c9fe62ec6d4</v>
       </c>
     </row>
     <row r="118">
@@ -4512,10 +4512,10 @@
         <v>117</v>
       </c>
       <c r="B118" t="str">
-        <v>CERT-F1521375</v>
+        <v>CERT-30AAA573</v>
       </c>
       <c r="C118" t="str">
-        <v>Kartik jaiswal</v>
+        <v>Lalita Sharma</v>
       </c>
       <c r="D118" t="str">
         <v>Quantum nexus</v>
@@ -4539,7 +4539,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K118" t="str">
-        <v>f1521375-a030-40f5-9c4a-ce9fbb6f6b90</v>
+        <v>30aaa573-64c0-4b9e-a34d-b7f48aa18bc9</v>
       </c>
     </row>
     <row r="119">
@@ -4547,25 +4547,25 @@
         <v>118</v>
       </c>
       <c r="B119" t="str">
-        <v>CERT-4ED0C48E</v>
+        <v>CERT-F24FFFDB</v>
       </c>
       <c r="C119" t="str">
-        <v>Don Abraham</v>
+        <v>Shubham Sarangi</v>
       </c>
       <c r="D119" t="str">
-        <v>Quantum nexus</v>
+        <v>NexisEdge</v>
       </c>
       <c r="E119" t="str">
-        <v>TEAM-2026-0045</v>
+        <v>TEAM-2026-0039</v>
       </c>
       <c r="F119" t="str">
-        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
+        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
       </c>
       <c r="G119" t="str">
-        <v>kartikjaiswal9565@gmail.com</v>
+        <v>teamnexisedge@gmail.com</v>
       </c>
       <c r="H119" t="str">
-        <v>+91 7828830654</v>
+        <v>+91 8093580951</v>
       </c>
       <c r="I119" t="str">
         <v>Verified</v>
@@ -4574,7 +4574,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K119" t="str">
-        <v>4ed0c48e-c48e-42de-9bc0-8c9fe62ec6d4</v>
+        <v>f24fffdb-00bf-4201-a476-534ebb1d9ede</v>
       </c>
     </row>
     <row r="120">
@@ -4582,25 +4582,25 @@
         <v>119</v>
       </c>
       <c r="B120" t="str">
-        <v>CERT-30AAA573</v>
+        <v>CERT-FEE03E86</v>
       </c>
       <c r="C120" t="str">
-        <v>Lalita Sharma</v>
+        <v>Suhana Mishra</v>
       </c>
       <c r="D120" t="str">
-        <v>Quantum nexus</v>
+        <v>NexisEdge</v>
       </c>
       <c r="E120" t="str">
-        <v>TEAM-2026-0045</v>
+        <v>TEAM-2026-0039</v>
       </c>
       <c r="F120" t="str">
-        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
+        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
       </c>
       <c r="G120" t="str">
-        <v>kartikjaiswal9565@gmail.com</v>
+        <v>teamnexisedge@gmail.com</v>
       </c>
       <c r="H120" t="str">
-        <v>+91 7828830654</v>
+        <v>+91 8093580951</v>
       </c>
       <c r="I120" t="str">
         <v>Verified</v>
@@ -4609,7 +4609,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K120" t="str">
-        <v>30aaa573-64c0-4b9e-a34d-b7f48aa18bc9</v>
+        <v>fee03e86-587d-48da-b79e-62dbe1e0e03a</v>
       </c>
     </row>
     <row r="121">
@@ -4617,10 +4617,10 @@
         <v>120</v>
       </c>
       <c r="B121" t="str">
-        <v>CERT-F24FFFDB</v>
+        <v>CERT-229540B4</v>
       </c>
       <c r="C121" t="str">
-        <v>Shubham Sarangi</v>
+        <v>Shadab Khan</v>
       </c>
       <c r="D121" t="str">
         <v>NexisEdge</v>
@@ -4644,7 +4644,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K121" t="str">
-        <v>f24fffdb-00bf-4201-a476-534ebb1d9ede</v>
+        <v>229540b4-4c2c-4ff2-b133-4fb911c37bae</v>
       </c>
     </row>
     <row r="122">
@@ -4652,25 +4652,25 @@
         <v>121</v>
       </c>
       <c r="B122" t="str">
-        <v>CERT-FEE03E86</v>
+        <v>CERT-4D761CE5</v>
       </c>
       <c r="C122" t="str">
-        <v>Suhana Mishra</v>
+        <v>Aman Dixit</v>
       </c>
       <c r="D122" t="str">
-        <v>NexisEdge</v>
+        <v>Syntax Error</v>
       </c>
       <c r="E122" t="str">
-        <v>TEAM-2026-0039</v>
+        <v>TEAM-2026-0050</v>
       </c>
       <c r="F122" t="str">
-        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
+        <v>Madhav Institute of Technology &amp; Science</v>
       </c>
       <c r="G122" t="str">
-        <v>teamnexisedge@gmail.com</v>
+        <v>itsaman911@gmail.com</v>
       </c>
       <c r="H122" t="str">
-        <v>+91 8093580951</v>
+        <v>+91 9691878855</v>
       </c>
       <c r="I122" t="str">
         <v>Verified</v>
@@ -4679,7 +4679,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K122" t="str">
-        <v>fee03e86-587d-48da-b79e-62dbe1e0e03a</v>
+        <v>4d761ce5-e329-4c55-bc85-acffeef302ea</v>
       </c>
     </row>
     <row r="123">
@@ -4687,25 +4687,25 @@
         <v>122</v>
       </c>
       <c r="B123" t="str">
-        <v>CERT-229540B4</v>
+        <v>CERT-AE892CBF</v>
       </c>
       <c r="C123" t="str">
-        <v>Shadab Khan</v>
+        <v>Parth Saxena</v>
       </c>
       <c r="D123" t="str">
-        <v>NexisEdge</v>
+        <v>Obsidian</v>
       </c>
       <c r="E123" t="str">
-        <v>TEAM-2026-0039</v>
+        <v>TEAM-2026-0042</v>
       </c>
       <c r="F123" t="str">
-        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
+        <v>Institute of Engineering and Science, IPS Academy (IES IPS), Indore</v>
       </c>
       <c r="G123" t="str">
-        <v>teamnexisedge@gmail.com</v>
+        <v>parthsaxena.tech@gmail.com</v>
       </c>
       <c r="H123" t="str">
-        <v>+91 8093580951</v>
+        <v>+91 9893890100</v>
       </c>
       <c r="I123" t="str">
         <v>Verified</v>
@@ -4714,7 +4714,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K123" t="str">
-        <v>229540b4-4c2c-4ff2-b133-4fb911c37bae</v>
+        <v>ae892cbf-7671-422f-9043-6e0800378573</v>
       </c>
     </row>
     <row r="124">
@@ -4722,25 +4722,25 @@
         <v>123</v>
       </c>
       <c r="B124" t="str">
-        <v>CERT-4D761CE5</v>
+        <v>CERT-B97EFCAA</v>
       </c>
       <c r="C124" t="str">
-        <v>Aman Dixit</v>
+        <v>Pranjal</v>
       </c>
       <c r="D124" t="str">
-        <v>Syntax Error</v>
+        <v>Obsidian</v>
       </c>
       <c r="E124" t="str">
-        <v>TEAM-2026-0050</v>
+        <v>TEAM-2026-0042</v>
       </c>
       <c r="F124" t="str">
-        <v>Madhav Institute of Technology &amp; Science</v>
+        <v>Institute of Engineering and Science, IPS Academy (IES IPS), Indore</v>
       </c>
       <c r="G124" t="str">
-        <v>itsaman911@gmail.com</v>
+        <v>parthsaxena.tech@gmail.com</v>
       </c>
       <c r="H124" t="str">
-        <v>+91 9691878855</v>
+        <v>+91 9893890100</v>
       </c>
       <c r="I124" t="str">
         <v>Verified</v>
@@ -4749,7 +4749,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K124" t="str">
-        <v>4d761ce5-e329-4c55-bc85-acffeef302ea</v>
+        <v>b97efcaa-a5d8-4f25-846e-63982f4c29a5</v>
       </c>
     </row>
     <row r="125">
@@ -4757,10 +4757,10 @@
         <v>124</v>
       </c>
       <c r="B125" t="str">
-        <v>CERT-AE892CBF</v>
+        <v>CERT-782FAAC6</v>
       </c>
       <c r="C125" t="str">
-        <v>Parth Saxena</v>
+        <v>Sanidhya Wankhede</v>
       </c>
       <c r="D125" t="str">
         <v>Obsidian</v>
@@ -4784,7 +4784,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K125" t="str">
-        <v>ae892cbf-7671-422f-9043-6e0800378573</v>
+        <v>782faac6-8214-4350-b254-4b90b574b134</v>
       </c>
     </row>
     <row r="126">
@@ -4792,25 +4792,25 @@
         <v>125</v>
       </c>
       <c r="B126" t="str">
-        <v>CERT-B97EFCAA</v>
+        <v>CERT-EF901E34</v>
       </c>
       <c r="C126" t="str">
-        <v>Pranjal</v>
+        <v>Divy Jain</v>
       </c>
       <c r="D126" t="str">
-        <v>Obsidian</v>
+        <v>ModelX</v>
       </c>
       <c r="E126" t="str">
-        <v>TEAM-2026-0042</v>
+        <v>TEAM-2026-0035</v>
       </c>
       <c r="F126" t="str">
         <v>Institute of Engineering and Science, IPS Academy (IES IPS), Indore</v>
       </c>
       <c r="G126" t="str">
-        <v>parthsaxena.tech@gmail.com</v>
+        <v>deepjain615@gmail.com</v>
       </c>
       <c r="H126" t="str">
-        <v>+91 9893890100</v>
+        <v>+91 9407573955</v>
       </c>
       <c r="I126" t="str">
         <v>Verified</v>
@@ -4819,7 +4819,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K126" t="str">
-        <v>b97efcaa-a5d8-4f25-846e-63982f4c29a5</v>
+        <v>ef901e34-17ec-4d13-aaca-50b25590164c</v>
       </c>
     </row>
     <row r="127">
@@ -4827,25 +4827,25 @@
         <v>126</v>
       </c>
       <c r="B127" t="str">
-        <v>CERT-782FAAC6</v>
+        <v>CERT-1615FB1E</v>
       </c>
       <c r="C127" t="str">
-        <v>Sanidhya Wankhede</v>
+        <v>Meet Jain</v>
       </c>
       <c r="D127" t="str">
-        <v>Obsidian</v>
+        <v>ModelX</v>
       </c>
       <c r="E127" t="str">
-        <v>TEAM-2026-0042</v>
+        <v>TEAM-2026-0035</v>
       </c>
       <c r="F127" t="str">
         <v>Institute of Engineering and Science, IPS Academy (IES IPS), Indore</v>
       </c>
       <c r="G127" t="str">
-        <v>parthsaxena.tech@gmail.com</v>
+        <v>deepjain615@gmail.com</v>
       </c>
       <c r="H127" t="str">
-        <v>+91 9893890100</v>
+        <v>+91 9407573955</v>
       </c>
       <c r="I127" t="str">
         <v>Verified</v>
@@ -4854,7 +4854,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K127" t="str">
-        <v>782faac6-8214-4350-b254-4b90b574b134</v>
+        <v>1615fb1e-3a6a-4c94-9106-a3f39d94a071</v>
       </c>
     </row>
     <row r="128">
@@ -4862,25 +4862,25 @@
         <v>127</v>
       </c>
       <c r="B128" t="str">
-        <v>CERT-EF901E34</v>
+        <v>CERT-1C803972</v>
       </c>
       <c r="C128" t="str">
-        <v>Divy Jain</v>
+        <v>Shivam Sharma</v>
       </c>
       <c r="D128" t="str">
-        <v>ModelX</v>
+        <v>Obsidian</v>
       </c>
       <c r="E128" t="str">
-        <v>TEAM-2026-0035</v>
+        <v>TEAM-2026-0042</v>
       </c>
       <c r="F128" t="str">
         <v>Institute of Engineering and Science, IPS Academy (IES IPS), Indore</v>
       </c>
       <c r="G128" t="str">
-        <v>deepjain615@gmail.com</v>
+        <v>parthsaxena.tech@gmail.com</v>
       </c>
       <c r="H128" t="str">
-        <v>+91 9407573955</v>
+        <v>+91 9893890100</v>
       </c>
       <c r="I128" t="str">
         <v>Verified</v>
@@ -4889,7 +4889,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K128" t="str">
-        <v>ef901e34-17ec-4d13-aaca-50b25590164c</v>
+        <v>1c803972-8ebf-437d-97a5-ad7f09700e9d</v>
       </c>
     </row>
     <row r="129">
@@ -4897,25 +4897,25 @@
         <v>128</v>
       </c>
       <c r="B129" t="str">
-        <v>CERT-1615FB1E</v>
+        <v>CERT-31B77768</v>
       </c>
       <c r="C129" t="str">
-        <v>Meet Jain</v>
+        <v>Ravikant Upadhyay</v>
       </c>
       <c r="D129" t="str">
-        <v>ModelX</v>
+        <v>NeuroStack</v>
       </c>
       <c r="E129" t="str">
-        <v>TEAM-2026-0035</v>
+        <v>TEAM-2026-0038</v>
       </c>
       <c r="F129" t="str">
-        <v>Institute of Engineering and Science, IPS Academy (IES IPS), Indore</v>
+        <v>Oriental Institute of Science and Technology</v>
       </c>
       <c r="G129" t="str">
-        <v>deepjain615@gmail.com</v>
+        <v>raaylucifer1@gmail.com</v>
       </c>
       <c r="H129" t="str">
-        <v>+91 9407573955</v>
+        <v>+91 8269908276</v>
       </c>
       <c r="I129" t="str">
         <v>Verified</v>
@@ -4924,7 +4924,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K129" t="str">
-        <v>1615fb1e-3a6a-4c94-9106-a3f39d94a071</v>
+        <v>31b77768-e0f0-4a70-8364-5ec37aa47681</v>
       </c>
     </row>
     <row r="130">
@@ -4932,25 +4932,25 @@
         <v>129</v>
       </c>
       <c r="B130" t="str">
-        <v>CERT-1C803972</v>
+        <v>CERT-D39D8C8C</v>
       </c>
       <c r="C130" t="str">
-        <v>Shivam Sharma</v>
+        <v>Kashish Kumari</v>
       </c>
       <c r="D130" t="str">
-        <v>Obsidian</v>
+        <v>NeuroStack</v>
       </c>
       <c r="E130" t="str">
-        <v>TEAM-2026-0042</v>
+        <v>TEAM-2026-0038</v>
       </c>
       <c r="F130" t="str">
-        <v>Institute of Engineering and Science, IPS Academy (IES IPS), Indore</v>
+        <v>Oriental Institute of Science and Technology</v>
       </c>
       <c r="G130" t="str">
-        <v>parthsaxena.tech@gmail.com</v>
+        <v>raaylucifer1@gmail.com</v>
       </c>
       <c r="H130" t="str">
-        <v>+91 9893890100</v>
+        <v>+91 8269908276</v>
       </c>
       <c r="I130" t="str">
         <v>Verified</v>
@@ -4959,7 +4959,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K130" t="str">
-        <v>1c803972-8ebf-437d-97a5-ad7f09700e9d</v>
+        <v>d39d8c8c-2239-4cbd-89a0-29dfb1f11c55</v>
       </c>
     </row>
     <row r="131">
@@ -4967,10 +4967,10 @@
         <v>130</v>
       </c>
       <c r="B131" t="str">
-        <v>CERT-31B77768</v>
+        <v>CERT-9B6A6661</v>
       </c>
       <c r="C131" t="str">
-        <v>Ravikant Upadhyay</v>
+        <v>Saksham Kumar Mishra</v>
       </c>
       <c r="D131" t="str">
         <v>NeuroStack</v>
@@ -4994,7 +4994,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K131" t="str">
-        <v>31b77768-e0f0-4a70-8364-5ec37aa47681</v>
+        <v>9b6a6661-ef1f-4b90-a147-3eff5a49868a</v>
       </c>
     </row>
     <row r="132">
@@ -5002,25 +5002,25 @@
         <v>131</v>
       </c>
       <c r="B132" t="str">
-        <v>CERT-D39D8C8C</v>
+        <v>CERT-37C32BE2</v>
       </c>
       <c r="C132" t="str">
-        <v>Kashish Kumari</v>
+        <v>Harsh Manmode</v>
       </c>
       <c r="D132" t="str">
-        <v>NeuroStack</v>
+        <v>SarthiX</v>
       </c>
       <c r="E132" t="str">
-        <v>TEAM-2026-0038</v>
+        <v>TEAM-2026-0047</v>
       </c>
       <c r="F132" t="str">
-        <v>Oriental Institute of Science and Technology</v>
+        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
       </c>
       <c r="G132" t="str">
-        <v>raaylucifer1@gmail.com</v>
+        <v>harshmanmode79@gmail.com</v>
       </c>
       <c r="H132" t="str">
-        <v>+91 8269908276</v>
+        <v>+91 8305721431</v>
       </c>
       <c r="I132" t="str">
         <v>Verified</v>
@@ -5029,7 +5029,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K132" t="str">
-        <v>d39d8c8c-2239-4cbd-89a0-29dfb1f11c55</v>
+        <v>37c32be2-43a4-46bb-97c7-6835899d6e10</v>
       </c>
     </row>
     <row r="133">
@@ -5037,25 +5037,25 @@
         <v>132</v>
       </c>
       <c r="B133" t="str">
-        <v>CERT-9B6A6661</v>
+        <v>CERT-BAE6A7CE</v>
       </c>
       <c r="C133" t="str">
-        <v>Saksham Kumar Mishra</v>
+        <v>Amit Manmode</v>
       </c>
       <c r="D133" t="str">
-        <v>NeuroStack</v>
+        <v>SarthiX</v>
       </c>
       <c r="E133" t="str">
-        <v>TEAM-2026-0038</v>
+        <v>TEAM-2026-0047</v>
       </c>
       <c r="F133" t="str">
-        <v>Oriental Institute of Science and Technology</v>
+        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
       </c>
       <c r="G133" t="str">
-        <v>raaylucifer1@gmail.com</v>
+        <v>harshmanmode79@gmail.com</v>
       </c>
       <c r="H133" t="str">
-        <v>+91 8269908276</v>
+        <v>+91 8305721431</v>
       </c>
       <c r="I133" t="str">
         <v>Verified</v>
@@ -5064,7 +5064,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K133" t="str">
-        <v>9b6a6661-ef1f-4b90-a147-3eff5a49868a</v>
+        <v>bae6a7ce-c860-44fa-bb01-490e51ec479b</v>
       </c>
     </row>
     <row r="134">
@@ -5072,10 +5072,10 @@
         <v>133</v>
       </c>
       <c r="B134" t="str">
-        <v>CERT-37C32BE2</v>
+        <v>CERT-34115E25</v>
       </c>
       <c r="C134" t="str">
-        <v>Harsh Manmode</v>
+        <v>Vivek Dahat</v>
       </c>
       <c r="D134" t="str">
         <v>SarthiX</v>
@@ -5099,7 +5099,7 @@
         <v>2026-09-12</v>
       </c>
       <c r="K134" t="str">
-        <v>37c32be2-43a4-46bb-97c7-6835899d6e10</v>
+        <v>34115e25-02d2-4f88-b64c-6f9ed2a6a482</v>
       </c>
     </row>
     <row r="135">
@@ -5107,34 +5107,34 @@
         <v>134</v>
       </c>
       <c r="B135" t="str">
-        <v>CERT-BAE6A7CE</v>
+        <v>CERT-0921DD78</v>
       </c>
       <c r="C135" t="str">
-        <v>Amit Manmode</v>
+        <v>Sanika Nikumbh</v>
       </c>
       <c r="D135" t="str">
-        <v>SarthiX</v>
+        <v>NeuroForge</v>
       </c>
       <c r="E135" t="str">
-        <v>TEAM-2026-0047</v>
+        <v>TEAM-2026-0037</v>
       </c>
       <c r="F135" t="str">
-        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
+        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
       </c>
       <c r="G135" t="str">
-        <v>harshmanmode79@gmail.com</v>
+        <v>teamnexisedge@gmail.com</v>
       </c>
       <c r="H135" t="str">
-        <v>+91 8305721431</v>
+        <v>+91 7875443935</v>
       </c>
       <c r="I135" t="str">
-        <v>Verified</v>
+        <v>Pending</v>
       </c>
       <c r="J135" t="str">
         <v>2026-09-12</v>
       </c>
       <c r="K135" t="str">
-        <v>bae6a7ce-c860-44fa-bb01-490e51ec479b</v>
+        <v>0921dd78-843b-4863-bfae-cb750327a492</v>
       </c>
     </row>
     <row r="136">
@@ -5142,34 +5142,34 @@
         <v>135</v>
       </c>
       <c r="B136" t="str">
-        <v>CERT-34115E25</v>
+        <v>CERT-3BA3C386</v>
       </c>
       <c r="C136" t="str">
-        <v>Vivek Dahat</v>
+        <v>Vaishnavi Mahadik</v>
       </c>
       <c r="D136" t="str">
-        <v>SarthiX</v>
+        <v>NeuroForge</v>
       </c>
       <c r="E136" t="str">
-        <v>TEAM-2026-0047</v>
+        <v>TEAM-2026-0037</v>
       </c>
       <c r="F136" t="str">
-        <v>Madhav Institute of Technology and Science (MITS), Gwalior</v>
+        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
       </c>
       <c r="G136" t="str">
-        <v>harshmanmode79@gmail.com</v>
+        <v>teamnexisedge@gmail.com</v>
       </c>
       <c r="H136" t="str">
-        <v>+91 8305721431</v>
+        <v>+91 7875443935</v>
       </c>
       <c r="I136" t="str">
-        <v>Verified</v>
+        <v>Pending</v>
       </c>
       <c r="J136" t="str">
         <v>2026-09-12</v>
       </c>
       <c r="K136" t="str">
-        <v>34115e25-02d2-4f88-b64c-6f9ed2a6a482</v>
+        <v>3ba3c386-3ba9-4294-8db8-a9d7cf9d5972</v>
       </c>
     </row>
     <row r="137">

</xml_diff>

<commit_message>
fix(neuroforge): update college name to Pune for NeuroForge
</commit_message>
<xml_diff>
--- a/hackathon_participants_certificate_ids.xlsx
+++ b/hackathon_participants_certificate_ids.xlsx
@@ -3684,7 +3684,7 @@
         <v>TEAM-2026-0037</v>
       </c>
       <c r="F94" t="str">
-        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
+        <v>Pune</v>
       </c>
       <c r="G94" t="str">
         <v>teamnexisedge@gmail.com</v>
@@ -4384,7 +4384,7 @@
         <v>TEAM-2026-0037</v>
       </c>
       <c r="F114" t="str">
-        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
+        <v>Pune</v>
       </c>
       <c r="G114" t="str">
         <v>teamnexisedge@gmail.com</v>
@@ -5119,7 +5119,7 @@
         <v>TEAM-2026-0037</v>
       </c>
       <c r="F135" t="str">
-        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
+        <v>Pune</v>
       </c>
       <c r="G135" t="str">
         <v>teamnexisedge@gmail.com</v>
@@ -5154,7 +5154,7 @@
         <v>TEAM-2026-0037</v>
       </c>
       <c r="F136" t="str">
-        <v>Trident Academy of Technology (TAT), Bhubaneswar</v>
+        <v>Pune</v>
       </c>
       <c r="G136" t="str">
         <v>teamnexisedge@gmail.com</v>

</xml_diff>